<commit_message>
Learn customer preferences from feedback and show next-ranked listing
- preference.py: online learning of criterion weights from rejects/likes,
  reason-driven boosts ("너무 비싸요" -> price), attribute likes/dislikes
  with protection for explicitly requested features; per-customer and
  office-wide models persisted in SQLite
- Session re-ranks remaining listings after each rejection so the next
  shown listing reflects what was learned
- Parser: '2억원대'/'200평대' bands, sunlight synonyms (채광/햇빛/일조),
  unspaced county names, notice when a non-land type is requested
- CLI: free-text replies route to next-rank or condition change, 'w'
  shows learned preferences; Eumseong sample listings; tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NxNSd6rzBRzEYPaCwTsUau
</commit_message>
<xml_diff>
--- a/sample_data/토지/토지매물장부_2026.xlsx
+++ b/sample_data/토지/토지매물장부_2026.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet name="양평" sheetId="1" r:id="rId1"/>
     <sheet name="여주" sheetId="2" r:id="rId2"/>
+    <sheet name="음성" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="153">
   <si>
     <t>양평 토지 매물 장부 (2026)</t>
   </si>
@@ -369,6 +370,111 @@
   </si>
   <si>
     <t>010-9090-1212</t>
+  </si>
+  <si>
+    <t>음성 토지 매물 장부 (2026)</t>
+  </si>
+  <si>
+    <t>E-3001</t>
+  </si>
+  <si>
+    <t>E-3002</t>
+  </si>
+  <si>
+    <t>E-3003</t>
+  </si>
+  <si>
+    <t>E-3004</t>
+  </si>
+  <si>
+    <t>E-3005</t>
+  </si>
+  <si>
+    <t>E-3006</t>
+  </si>
+  <si>
+    <t>충청북도 음성군 금왕읍 무극리 210-3</t>
+  </si>
+  <si>
+    <t>충청북도 음성군 대소면 오류리 55</t>
+  </si>
+  <si>
+    <t>충청북도 음성군 음성읍 평곡리 8-1</t>
+  </si>
+  <si>
+    <t>충청북도 음성군 감곡면 오향리 301</t>
+  </si>
+  <si>
+    <t>충청북도 음성군 원남면 하당리 77</t>
+  </si>
+  <si>
+    <t>충청북도 음성군 맹동면 쌍정리 12-4</t>
+  </si>
+  <si>
+    <t>2억 3천만원</t>
+  </si>
+  <si>
+    <t>2억 7천</t>
+  </si>
+  <si>
+    <t>2억 9천</t>
+  </si>
+  <si>
+    <t>1억 8천</t>
+  </si>
+  <si>
+    <t>2억 4천</t>
+  </si>
+  <si>
+    <t>2026-10-02</t>
+  </si>
+  <si>
+    <t>2026-09-15</t>
+  </si>
+  <si>
+    <t>2026-08-20</t>
+  </si>
+  <si>
+    <t>2026-09-28</t>
+  </si>
+  <si>
+    <t>2026-07-30</t>
+  </si>
+  <si>
+    <t>2026-10-06</t>
+  </si>
+  <si>
+    <t>정남향 평지, 채광 우수, 금왕IC 5분</t>
+  </si>
+  <si>
+    <t>남동향 완경사, 햇빛 잘 듦, 전원주택 부지</t>
+  </si>
+  <si>
+    <t>북향, 뒤로 산이 있어 오후 그늘</t>
+  </si>
+  <si>
+    <t>창고 부지, 대형차 진입, 채광 양호</t>
+  </si>
+  <si>
+    <t>남향 밭, 마을 인접</t>
+  </si>
+  <si>
+    <t>혁신도시 인근, 동향, 상가 밀집</t>
+  </si>
+  <si>
+    <t>010-3131-4242</t>
+  </si>
+  <si>
+    <t>010-3232-4343</t>
+  </si>
+  <si>
+    <t>010-3434-4545</t>
+  </si>
+  <si>
+    <t>010-3535-4646</t>
+  </si>
+  <si>
+    <t>010-3636-4747</t>
   </si>
 </sst>
 </file>
@@ -1265,4 +1371,264 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J3" t="s">
+        <v>71</v>
+      </c>
+      <c r="K3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4">
+        <v>826</v>
+      </c>
+      <c r="F4" t="s">
+        <v>131</v>
+      </c>
+      <c r="G4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I4" t="s">
+        <v>136</v>
+      </c>
+      <c r="J4" t="s">
+        <v>142</v>
+      </c>
+      <c r="K4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" t="s">
+        <v>126</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5">
+        <v>1157</v>
+      </c>
+      <c r="F5" t="s">
+        <v>132</v>
+      </c>
+      <c r="G5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H5" t="s">
+        <v>58</v>
+      </c>
+      <c r="I5" t="s">
+        <v>137</v>
+      </c>
+      <c r="J5" t="s">
+        <v>143</v>
+      </c>
+      <c r="K5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6">
+        <v>661</v>
+      </c>
+      <c r="F6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G6" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" t="s">
+        <v>58</v>
+      </c>
+      <c r="I6" t="s">
+        <v>138</v>
+      </c>
+      <c r="J6" t="s">
+        <v>144</v>
+      </c>
+      <c r="K6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7">
+        <v>1983</v>
+      </c>
+      <c r="F7" t="s">
+        <v>133</v>
+      </c>
+      <c r="G7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" t="s">
+        <v>58</v>
+      </c>
+      <c r="I7" t="s">
+        <v>139</v>
+      </c>
+      <c r="J7" t="s">
+        <v>145</v>
+      </c>
+      <c r="K7" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8">
+        <v>1322</v>
+      </c>
+      <c r="F8" t="s">
+        <v>134</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" t="s">
+        <v>140</v>
+      </c>
+      <c r="J8" t="s">
+        <v>146</v>
+      </c>
+      <c r="K8" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B9" t="s">
+        <v>130</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9">
+        <v>562</v>
+      </c>
+      <c r="F9" t="s">
+        <v>135</v>
+      </c>
+      <c r="G9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H9" t="s">
+        <v>58</v>
+      </c>
+      <c r="I9" t="s">
+        <v>141</v>
+      </c>
+      <c r="J9" t="s">
+        <v>147</v>
+      </c>
+      <c r="K9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>